<commit_message>
update end member table
</commit_message>
<xml_diff>
--- a/data/PO14C.xlsx
+++ b/data/PO14C.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Sarah\Dropbox\Shakil_Thesisdrafts\Chapter3\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sarah Shakil\Documents\PhD_Ch3\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89ADA08E-BA4F-4B16-AF8D-7C04728A7448}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE9165E-0694-4699-A1A4-C1D69AF4ECD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3345" yWindow="660" windowWidth="23445" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="25470" windowHeight="13980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PO14C" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="PO14C">PO14C!$A$1:$Y$53</definedName>
   </definedNames>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="143">
   <si>
     <t>Slump Site</t>
   </si>
@@ -440,6 +453,18 @@
   </si>
   <si>
     <t>dist</t>
+  </si>
+  <si>
+    <t>CB</t>
+  </si>
+  <si>
+    <t>Wilson</t>
+  </si>
+  <si>
+    <t>From Lacele et al. 2019 JGR-Biogeosciences - Table1-CBsite-unit2ishol-unit3iaple</t>
+  </si>
+  <si>
+    <t>From Lacele et al. 2019 JGR-Biogeosciences - Table1-Wilsonsite-unit2ishol-unit3iaple</t>
   </si>
 </sst>
 </file>
@@ -477,7 +502,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -498,9 +523,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -538,9 +563,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -573,26 +598,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -625,26 +633,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -818,11 +809,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y53"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
@@ -3997,6 +3990,168 @@
         <v>29</v>
       </c>
     </row>
+    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>139</v>
+      </c>
+      <c r="B54" t="s">
+        <v>51</v>
+      </c>
+      <c r="C54" t="s">
+        <v>55</v>
+      </c>
+      <c r="H54" t="s">
+        <v>31</v>
+      </c>
+      <c r="J54">
+        <v>24494</v>
+      </c>
+      <c r="K54">
+        <v>127</v>
+      </c>
+      <c r="L54">
+        <f>EXP((J54/-8033))</f>
+        <v>4.7398146007110162E-2</v>
+      </c>
+      <c r="Y54" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="55" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>139</v>
+      </c>
+      <c r="B55" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" t="s">
+        <v>55</v>
+      </c>
+      <c r="H55" t="s">
+        <v>31</v>
+      </c>
+      <c r="J55">
+        <v>38367</v>
+      </c>
+      <c r="K55">
+        <v>480</v>
+      </c>
+      <c r="L55">
+        <f t="shared" ref="L55:L59" si="0">EXP((J55/-8033))</f>
+        <v>8.4281896139422711E-3</v>
+      </c>
+      <c r="Y55" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>139</v>
+      </c>
+      <c r="B56" t="s">
+        <v>51</v>
+      </c>
+      <c r="C56" t="s">
+        <v>61</v>
+      </c>
+      <c r="H56" t="s">
+        <v>31</v>
+      </c>
+      <c r="J56">
+        <v>40397</v>
+      </c>
+      <c r="K56">
+        <v>758</v>
+      </c>
+      <c r="L56">
+        <f t="shared" si="0"/>
+        <v>6.5461324693198092E-3</v>
+      </c>
+      <c r="Y56" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>139</v>
+      </c>
+      <c r="B57" t="s">
+        <v>51</v>
+      </c>
+      <c r="C57" t="s">
+        <v>61</v>
+      </c>
+      <c r="H57" t="s">
+        <v>31</v>
+      </c>
+      <c r="J57">
+        <v>39318</v>
+      </c>
+      <c r="K57">
+        <v>582</v>
+      </c>
+      <c r="L57">
+        <f t="shared" si="0"/>
+        <v>7.4872033158925174E-3</v>
+      </c>
+      <c r="Y57" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58" t="s">
+        <v>51</v>
+      </c>
+      <c r="C58" t="s">
+        <v>55</v>
+      </c>
+      <c r="H58" t="s">
+        <v>31</v>
+      </c>
+      <c r="J58">
+        <v>39398</v>
+      </c>
+      <c r="K58">
+        <v>719</v>
+      </c>
+      <c r="L58">
+        <f t="shared" si="0"/>
+        <v>7.4130089223205789E-3</v>
+      </c>
+      <c r="Y58" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" t="s">
+        <v>61</v>
+      </c>
+      <c r="H59" t="s">
+        <v>31</v>
+      </c>
+      <c r="J59">
+        <v>43603</v>
+      </c>
+      <c r="K59">
+        <v>885</v>
+      </c>
+      <c r="L59">
+        <f t="shared" si="0"/>
+        <v>4.3919385611812219E-3</v>
+      </c>
+      <c r="Y59" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>